<commit_message>
update on excel emport
</commit_message>
<xml_diff>
--- a/templates/PURCHASE_JOURNAL_TEMPLATE.xlsx
+++ b/templates/PURCHASE_JOURNAL_TEMPLATE.xlsx
@@ -1,35 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29505"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\dloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97443657-71B2-4406-96BC-40E26A6318DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{9ED0BF36-3A4D-4022-AB9B-70DAE7955819}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="August" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
-  </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="_xlcn.WorksheetConnection_Sheet1A1H5111" hidden="1">[1]CD!$B$1:$I$144</definedName>
-    <definedName name="PurchaseRecord">#REF!</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+  <ns0:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29505"/>
+  <ns0:workbookPr defaultThemeVersion="166925"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="F:\dloads\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97443657-71B2-4406-96BC-40E26A6318DC}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns0:bookViews>
+    <ns0:workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" ns6:uid="{9ED0BF36-3A4D-4022-AB9B-70DAE7955819}"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="August" sheetId="2" ns7:id="rId1"/>
+    <ns0:sheet name="Sheet1" sheetId="1" ns7:id="rId2"/>
+  </ns0:sheets>
+  <ns0:definedNames/>
+  <ns0:extLst>
+    <ns0:ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns8:workbookPr chartTrackingRefBase="1"/>
+    </ns0:ext>
+  </ns0:extLst>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1284,19 +1277,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="CD"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>